<commit_message>
fix(products): align xlsx templates and export headers with UI column names
- Rename first-column header: "name" -> "product" (catalog) / "dish" (menu)
  to match UI labels (Producto/Product/Prodotto vs Plato/Dish/Piatto)
- Update export CSV headers to match templates (round-trip safe)
- Add product/dish/plato/piatto/plat/produkt/prodotto/produit as
  import-parser aliases so existing sheets still import correctly
- Fix toggleAvailable sending stock_qty:1 on enable, which triggered
  the low-stock banner (<=5) spuriously — now only sends is_available
- Add truncate+title to menu description cell; add maxlength=500 to
  description textarea
- Regenerate catalog_template.xlsx and menu_template.xlsx
</commit_message>
<xml_diff>
--- a/public/catalog_template.xlsx
+++ b/public/catalog_template.xlsx
@@ -15,7 +15,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="52">
   <si>
-    <t>name</t>
+    <t>product</t>
   </si>
   <si>
     <t>category</t>
@@ -96,7 +96,7 @@
     <t>Columns</t>
   </si>
   <si>
-    <t>name (required) — the name customers see and search for.</t>
+    <t>product (required) — the name customers see and search for.</t>
   </si>
   <si>
     <t>category — used to group items (e.g. Bouquets, Starters). Optional but recommended.</t>
@@ -141,7 +141,7 @@
     <t>Columnas</t>
   </si>
   <si>
-    <t>name (obligatorio) — el nombre que ven y buscan los clientes.</t>
+    <t>product (obligatorio) — el nombre que ven y buscan los clientes.</t>
   </si>
   <si>
     <t>category — agrupa los ítems (ej: Ramos, Entradas). Opcional pero recomendado.</t>

</xml_diff>